<commit_message>
CONSAÚDE: paleta própria (grafite e vinho) na planilha de vícios e no deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrfDHY9D3MKaQfyrVNihp9
</commit_message>
<xml_diff>
--- a/concessoes/consaude-conc-2026/output/2026_10_08_CONSAUDE_Vicios_identificados.xlsx
+++ b/concessoes/consaude-conc-2026/output/2026_10_08_CONSAUDE_Vicios_identificados.xlsx
@@ -45,7 +45,7 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
-      <color rgb="FF00B0F0"/>
+      <color rgb="FF8C2F39"/>
       <sz val="12"/>
     </font>
     <font>
@@ -67,7 +67,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor rgb="FF2E3236"/>
       </patternFill>
     </fill>
   </fills>
@@ -528,7 +528,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="16"/>
             </rPr>
             <t>Edital nº [•]/2026 | Consórcio Intermunicipal de Saúde do Vale do Ribeira e Litoral Sul (CONSAÚDE)</t>
@@ -601,7 +601,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Bens reversíveis
@@ -622,7 +622,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -639,7 +639,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -656,7 +656,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -695,7 +695,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Disposição final
@@ -716,7 +716,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -733,7 +733,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -750,7 +750,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -788,7 +788,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -809,7 +809,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -826,7 +826,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -843,7 +843,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -860,7 +860,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -902,7 +902,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -923,7 +923,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -940,7 +940,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -957,7 +957,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -974,7 +974,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -991,7 +991,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1032,7 +1032,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -1053,7 +1053,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1070,7 +1070,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1087,7 +1087,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1104,7 +1104,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1147,7 +1147,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Matriz de riscos
@@ -1168,7 +1168,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1185,7 +1185,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1222,7 +1222,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Modelagem
@@ -1243,7 +1243,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1260,7 +1260,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1277,7 +1277,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1316,7 +1316,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -1337,7 +1337,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1354,7 +1354,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1371,7 +1371,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1388,7 +1388,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1427,7 +1427,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Inadimplência
@@ -1448,7 +1448,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1465,7 +1465,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1482,7 +1482,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1522,7 +1522,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Proteção de dados
@@ -1543,7 +1543,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1560,7 +1560,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1577,7 +1577,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1615,7 +1615,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Metas de desempenho
@@ -1636,7 +1636,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1653,7 +1653,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1670,7 +1670,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1687,7 +1687,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1704,7 +1704,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1744,7 +1744,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Metas de desempenho
@@ -1765,7 +1765,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1782,7 +1782,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1799,7 +1799,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1836,7 +1836,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">PIGIRS
@@ -1857,7 +1857,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1874,7 +1874,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1891,7 +1891,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1908,7 +1908,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1947,7 +1947,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Cronograma
@@ -1968,7 +1968,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1985,7 +1985,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2002,7 +2002,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2042,7 +2042,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Modelagem
@@ -2063,7 +2063,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2080,7 +2080,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2117,7 +2117,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Aspectos tributários
@@ -2138,7 +2138,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2155,7 +2155,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2172,7 +2172,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2189,7 +2189,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2228,7 +2228,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Matriz de riscos
@@ -2249,7 +2249,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2266,7 +2266,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2283,7 +2283,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2322,7 +2322,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -2343,7 +2343,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2360,7 +2360,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2399,7 +2399,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -2420,7 +2420,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2437,7 +2437,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2454,7 +2454,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2492,7 +2492,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Visita técnica
@@ -2513,7 +2513,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2530,7 +2530,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2569,7 +2569,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação econômico-financeira
@@ -2590,7 +2590,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2607,7 +2607,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2624,7 +2624,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2662,7 +2662,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação econômico-financeira
@@ -2683,7 +2683,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2700,7 +2700,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2717,7 +2717,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2755,7 +2755,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Habilitação
@@ -2776,7 +2776,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2793,7 +2793,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2831,7 +2831,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Documentos de habilitação
@@ -2852,7 +2852,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2869,7 +2869,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2907,7 +2907,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Garantia de execução
@@ -2928,7 +2928,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2945,7 +2945,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2962,7 +2962,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3000,7 +3000,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Inconsistências internas
@@ -3021,7 +3021,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3038,7 +3038,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3076,7 +3076,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Inconsistências internas
@@ -3097,7 +3097,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3134,7 +3134,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Documentos não disponibilizados
@@ -3155,7 +3155,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3172,7 +3172,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3189,7 +3189,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3272,7 +3272,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="16"/>
             </rPr>
             <t>Reservas estratégicas – não protocolar | uso interno</t>
@@ -3345,7 +3345,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -3366,7 +3366,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3383,7 +3383,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3400,7 +3400,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3438,7 +3438,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -3459,7 +3459,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3476,7 +3476,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3514,7 +3514,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Condições de assinatura
@@ -3535,7 +3535,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3552,7 +3552,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3590,7 +3590,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -3611,7 +3611,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3650,7 +3650,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Receitas acessórias
@@ -3671,7 +3671,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3688,7 +3688,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3726,7 +3726,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Metas de desempenho
@@ -3747,7 +3747,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3784,7 +3784,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Rota tecnológica
@@ -3805,7 +3805,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3822,7 +3822,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF00B0F0"/>
+              <color rgb="FF8C2F39"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>

</xml_diff>

<commit_message>
CONSAÚDE: identidade verde e branca na planilha de vícios e no deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrfDHY9D3MKaQfyrVNihp9
</commit_message>
<xml_diff>
--- a/concessoes/consaude-conc-2026/output/2026_10_08_CONSAUDE_Vicios_identificados.xlsx
+++ b/concessoes/consaude-conc-2026/output/2026_10_08_CONSAUDE_Vicios_identificados.xlsx
@@ -45,7 +45,7 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
-      <color rgb="FF8C2F39"/>
+      <color rgb="FF00703C"/>
       <sz val="12"/>
     </font>
     <font>
@@ -67,7 +67,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E3236"/>
+        <fgColor rgb="FF006237"/>
       </patternFill>
     </fill>
   </fills>
@@ -528,7 +528,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="16"/>
             </rPr>
             <t>Edital nº [•]/2026 | Consórcio Intermunicipal de Saúde do Vale do Ribeira e Litoral Sul (CONSAÚDE)</t>
@@ -601,7 +601,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Bens reversíveis
@@ -622,7 +622,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -639,7 +639,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -656,7 +656,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -695,7 +695,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Disposição final
@@ -716,7 +716,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -733,7 +733,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -750,7 +750,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -788,7 +788,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -809,7 +809,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -826,7 +826,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -843,7 +843,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -860,7 +860,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -902,7 +902,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -923,7 +923,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -940,7 +940,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -957,7 +957,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -974,7 +974,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -991,7 +991,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1032,7 +1032,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -1053,7 +1053,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1070,7 +1070,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1087,7 +1087,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1104,7 +1104,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1147,7 +1147,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Matriz de riscos
@@ -1168,7 +1168,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1185,7 +1185,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1222,7 +1222,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Modelagem
@@ -1243,7 +1243,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1260,7 +1260,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1277,7 +1277,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1316,7 +1316,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -1337,7 +1337,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1354,7 +1354,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1371,7 +1371,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1388,7 +1388,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1427,7 +1427,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Inadimplência
@@ -1448,7 +1448,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1465,7 +1465,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1482,7 +1482,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1522,7 +1522,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Proteção de dados
@@ -1543,7 +1543,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1560,7 +1560,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1577,7 +1577,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1615,7 +1615,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Metas de desempenho
@@ -1636,7 +1636,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1653,7 +1653,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1670,7 +1670,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1687,7 +1687,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1704,7 +1704,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1744,7 +1744,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Metas de desempenho
@@ -1765,7 +1765,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1782,7 +1782,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1799,7 +1799,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1836,7 +1836,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">PIGIRS
@@ -1857,7 +1857,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1874,7 +1874,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1891,7 +1891,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1908,7 +1908,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1947,7 +1947,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Cronograma
@@ -1968,7 +1968,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -1985,7 +1985,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2002,7 +2002,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2042,7 +2042,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Modelagem
@@ -2063,7 +2063,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2080,7 +2080,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2117,7 +2117,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Aspectos tributários
@@ -2138,7 +2138,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2155,7 +2155,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2172,7 +2172,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2189,7 +2189,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2228,7 +2228,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Matriz de riscos
@@ -2249,7 +2249,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2266,7 +2266,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2283,7 +2283,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2322,7 +2322,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -2343,7 +2343,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2360,7 +2360,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2399,7 +2399,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -2420,7 +2420,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2437,7 +2437,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2454,7 +2454,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2492,7 +2492,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Visita técnica
@@ -2513,7 +2513,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2530,7 +2530,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2569,7 +2569,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação econômico-financeira
@@ -2590,7 +2590,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2607,7 +2607,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2624,7 +2624,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2662,7 +2662,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação econômico-financeira
@@ -2683,7 +2683,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2700,7 +2700,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2717,7 +2717,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2755,7 +2755,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Habilitação
@@ -2776,7 +2776,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2793,7 +2793,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2831,7 +2831,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Documentos de habilitação
@@ -2852,7 +2852,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2869,7 +2869,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2907,7 +2907,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Garantia de execução
@@ -2928,7 +2928,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2945,7 +2945,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -2962,7 +2962,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3000,7 +3000,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Inconsistências internas
@@ -3021,7 +3021,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3038,7 +3038,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3076,7 +3076,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Inconsistências internas
@@ -3097,7 +3097,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3134,7 +3134,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Documentos não disponibilizados
@@ -3155,7 +3155,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3172,7 +3172,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3189,7 +3189,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3272,7 +3272,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="16"/>
             </rPr>
             <t>Reservas estratégicas – não protocolar | uso interno</t>
@@ -3345,7 +3345,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -3366,7 +3366,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3383,7 +3383,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3400,7 +3400,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3438,7 +3438,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Qualificação técnica
@@ -3459,7 +3459,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3476,7 +3476,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3514,7 +3514,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Condições de assinatura
@@ -3535,7 +3535,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3552,7 +3552,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3590,7 +3590,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Estrutura tarifária
@@ -3611,7 +3611,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3650,7 +3650,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Receitas acessórias
@@ -3671,7 +3671,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3688,7 +3688,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3726,7 +3726,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Metas de desempenho
@@ -3747,7 +3747,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3784,7 +3784,7 @@
             <rPr>
               <rFont val="Aptos"/>
               <b val="1"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t xml:space="preserve">Rota tecnológica
@@ -3805,7 +3805,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>
@@ -3822,7 +3822,7 @@
           <r>
             <rPr>
               <rFont val="Aptos"/>
-              <color rgb="FF8C2F39"/>
+              <color rgb="FF00703C"/>
               <sz val="12"/>
             </rPr>
             <t>•</t>

</xml_diff>